<commit_message>
added phase07 reg stages
</commit_message>
<xml_diff>
--- a/05_Snowflake_Advance_DE_Certificate/Domain_Wise_Flow_Lost.xlsx
+++ b/05_Snowflake_Advance_DE_Certificate/Domain_Wise_Flow_Lost.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Snowflake_Advance_Data_Engineering\05_Snowflake_Advance_DE_Certificate\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F14689AB-923A-4073-B501-7E9CFA7E32CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{66356C77-D32E-4BD7-BA6F-D59DEA1C42D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1273,7 +1273,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1295,6 +1295,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.39997558519241921"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1363,7 +1369,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1387,6 +1393,12 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1705,13 +1717,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13">
-      <c r="A1" s="9" t="s">
+      <c r="A1" s="11" t="s">
         <v>42</v>
       </c>
-      <c r="B1" s="9"/>
-      <c r="C1" s="9"/>
-      <c r="D1" s="9"/>
-      <c r="E1" s="9"/>
+      <c r="B1" s="11"/>
+      <c r="C1" s="11"/>
+      <c r="D1" s="11"/>
+      <c r="E1" s="11"/>
     </row>
     <row r="2" spans="1:13">
       <c r="A2" s="5" t="s">
@@ -1867,30 +1879,30 @@
       </c>
     </row>
     <row r="15" spans="1:13">
-      <c r="I15" s="14" t="s">
+      <c r="I15" s="16" t="s">
         <v>239</v>
       </c>
-      <c r="J15" s="14"/>
-      <c r="K15" s="14"/>
-      <c r="L15" s="14"/>
-      <c r="M15" s="14"/>
+      <c r="J15" s="16"/>
+      <c r="K15" s="16"/>
+      <c r="L15" s="16"/>
+      <c r="M15" s="16"/>
     </row>
     <row r="16" spans="1:13">
-      <c r="A16" s="10" t="s">
+      <c r="A16" s="12" t="s">
         <v>83</v>
       </c>
-      <c r="B16" s="11"/>
-      <c r="C16" s="12"/>
-      <c r="E16" s="10" t="s">
+      <c r="B16" s="13"/>
+      <c r="C16" s="14"/>
+      <c r="E16" s="12" t="s">
         <v>84</v>
       </c>
-      <c r="F16" s="11"/>
-      <c r="G16" s="12"/>
-      <c r="I16" s="14"/>
-      <c r="J16" s="14"/>
-      <c r="K16" s="14"/>
-      <c r="L16" s="14"/>
-      <c r="M16" s="14"/>
+      <c r="F16" s="13"/>
+      <c r="G16" s="14"/>
+      <c r="I16" s="16"/>
+      <c r="J16" s="16"/>
+      <c r="K16" s="16"/>
+      <c r="L16" s="16"/>
+      <c r="M16" s="16"/>
     </row>
     <row r="17" spans="1:13">
       <c r="A17" s="5" t="s">
@@ -1937,13 +1949,13 @@
       <c r="C18" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="E18" s="3">
+      <c r="E18" s="9">
         <v>1</v>
       </c>
-      <c r="F18" s="4" t="s">
+      <c r="F18" s="10" t="s">
         <v>87</v>
       </c>
-      <c r="G18" s="3" t="s">
+      <c r="G18" s="9" t="s">
         <v>8</v>
       </c>
       <c r="I18" s="1" t="s">
@@ -1970,13 +1982,13 @@
       <c r="C19" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="E19" s="3">
+      <c r="E19" s="9">
         <v>2</v>
       </c>
-      <c r="F19" s="4" t="s">
+      <c r="F19" s="10" t="s">
         <v>88</v>
       </c>
-      <c r="G19" s="3" t="s">
+      <c r="G19" s="9" t="s">
         <v>8</v>
       </c>
       <c r="I19" s="1" t="s">
@@ -2003,13 +2015,13 @@
       <c r="C20" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="E20" s="3">
+      <c r="E20" s="9">
         <v>3</v>
       </c>
-      <c r="F20" s="4" t="s">
+      <c r="F20" s="10" t="s">
         <v>89</v>
       </c>
-      <c r="G20" s="3" t="s">
+      <c r="G20" s="9" t="s">
         <v>8</v>
       </c>
       <c r="I20" s="1" t="s">
@@ -2038,13 +2050,13 @@
       <c r="C21" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="E21" s="3">
+      <c r="E21" s="9">
         <v>4</v>
       </c>
-      <c r="F21" s="4" t="s">
+      <c r="F21" s="10" t="s">
         <v>90</v>
       </c>
-      <c r="G21" s="3" t="s">
+      <c r="G21" s="9" t="s">
         <v>8</v>
       </c>
       <c r="I21" s="1" t="s">
@@ -2071,13 +2083,13 @@
       <c r="C22" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="E22" s="3">
+      <c r="E22" s="9">
         <v>5</v>
       </c>
-      <c r="F22" s="4" t="s">
+      <c r="F22" s="10" t="s">
         <v>91</v>
       </c>
-      <c r="G22" s="3" t="s">
+      <c r="G22" s="9" t="s">
         <v>8</v>
       </c>
       <c r="I22" s="1" t="s">
@@ -2104,13 +2116,13 @@
       <c r="C23" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="E23" s="3">
+      <c r="E23" s="9">
         <v>6</v>
       </c>
-      <c r="F23" s="4" t="s">
+      <c r="F23" s="10" t="s">
         <v>92</v>
       </c>
-      <c r="G23" s="3" t="s">
+      <c r="G23" s="9" t="s">
         <v>8</v>
       </c>
       <c r="I23" s="1" t="s">
@@ -2137,13 +2149,13 @@
       <c r="C24" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="E24" s="3">
+      <c r="E24" s="9">
         <v>7</v>
       </c>
-      <c r="F24" s="4" t="s">
+      <c r="F24" s="9" t="s">
         <v>93</v>
       </c>
-      <c r="G24" s="3" t="s">
+      <c r="G24" s="9" t="s">
         <v>8</v>
       </c>
       <c r="I24" s="1" t="s">
@@ -2172,13 +2184,13 @@
       <c r="C25" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="E25" s="3">
-        <v>8</v>
-      </c>
-      <c r="F25" s="4" t="s">
+      <c r="E25" s="9">
+        <v>8</v>
+      </c>
+      <c r="F25" s="9" t="s">
         <v>94</v>
       </c>
-      <c r="G25" s="3" t="s">
+      <c r="G25" s="9" t="s">
         <v>8</v>
       </c>
       <c r="I25" s="1" t="s">
@@ -2205,13 +2217,13 @@
       <c r="C26" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="E26" s="3">
+      <c r="E26" s="9">
         <v>9</v>
       </c>
-      <c r="F26" s="4" t="s">
+      <c r="F26" s="9" t="s">
         <v>95</v>
       </c>
-      <c r="G26" s="3" t="s">
+      <c r="G26" s="9" t="s">
         <v>8</v>
       </c>
       <c r="I26" s="1" t="s">
@@ -2238,13 +2250,13 @@
       <c r="C27" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="E27" s="3">
+      <c r="E27" s="9">
         <v>10</v>
       </c>
-      <c r="F27" s="4" t="s">
+      <c r="F27" s="9" t="s">
         <v>96</v>
       </c>
-      <c r="G27" s="3" t="s">
+      <c r="G27" s="9" t="s">
         <v>8</v>
       </c>
       <c r="I27" s="1" t="s">
@@ -2273,13 +2285,13 @@
       <c r="C28" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="E28" s="3">
+      <c r="E28" s="9">
         <v>11</v>
       </c>
-      <c r="F28" s="4" t="s">
+      <c r="F28" s="9" t="s">
         <v>97</v>
       </c>
-      <c r="G28" s="3" t="s">
+      <c r="G28" s="9" t="s">
         <v>8</v>
       </c>
       <c r="I28" s="1" t="s">
@@ -2306,13 +2318,13 @@
       <c r="C29" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="E29" s="3">
+      <c r="E29" s="9">
         <v>12</v>
       </c>
-      <c r="F29" s="4" t="s">
+      <c r="F29" s="9" t="s">
         <v>98</v>
       </c>
-      <c r="G29" s="3" t="s">
+      <c r="G29" s="9" t="s">
         <v>8</v>
       </c>
       <c r="I29" s="1" t="s">
@@ -2339,13 +2351,13 @@
       <c r="C30" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="E30" s="3">
+      <c r="E30" s="9">
         <v>13</v>
       </c>
-      <c r="F30" s="4" t="s">
+      <c r="F30" s="9" t="s">
         <v>99</v>
       </c>
-      <c r="G30" s="3" t="s">
+      <c r="G30" s="9" t="s">
         <v>8</v>
       </c>
       <c r="I30" s="1" t="s">
@@ -2372,13 +2384,13 @@
       <c r="C31" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="E31" s="3">
+      <c r="E31" s="9">
         <v>14</v>
       </c>
-      <c r="F31" s="4" t="s">
+      <c r="F31" s="9" t="s">
         <v>100</v>
       </c>
-      <c r="G31" s="3" t="s">
+      <c r="G31" s="9" t="s">
         <v>8</v>
       </c>
       <c r="I31" s="1" t="s">
@@ -2405,13 +2417,13 @@
       <c r="C32" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="E32" s="3">
+      <c r="E32" s="9">
         <v>15</v>
       </c>
-      <c r="F32" s="4" t="s">
+      <c r="F32" s="9" t="s">
         <v>101</v>
       </c>
-      <c r="G32" s="3" t="s">
+      <c r="G32" s="9" t="s">
         <v>8</v>
       </c>
     </row>
@@ -2923,20 +2935,20 @@
       </c>
     </row>
     <row r="69" spans="1:5">
-      <c r="A69" s="13" t="s">
+      <c r="A69" s="15" t="s">
         <v>199</v>
       </c>
-      <c r="B69" s="13"/>
-      <c r="C69" s="13"/>
-      <c r="D69" s="13"/>
-      <c r="E69" s="13"/>
+      <c r="B69" s="15"/>
+      <c r="C69" s="15"/>
+      <c r="D69" s="15"/>
+      <c r="E69" s="15"/>
     </row>
     <row r="70" spans="1:5">
-      <c r="A70" s="13"/>
-      <c r="B70" s="13"/>
-      <c r="C70" s="13"/>
-      <c r="D70" s="13"/>
-      <c r="E70" s="13"/>
+      <c r="A70" s="15"/>
+      <c r="B70" s="15"/>
+      <c r="C70" s="15"/>
+      <c r="D70" s="15"/>
+      <c r="E70" s="15"/>
     </row>
     <row r="71" spans="1:5">
       <c r="A71" s="7" t="s">
@@ -3212,13 +3224,13 @@
   <sheetFormatPr defaultColWidth="35.77734375" defaultRowHeight="14.4"/>
   <sheetData>
     <row r="1" spans="1:7">
-      <c r="A1" s="9" t="s">
+      <c r="A1" s="11" t="s">
         <v>42</v>
       </c>
-      <c r="B1" s="9"/>
-      <c r="C1" s="9"/>
-      <c r="D1" s="9"/>
-      <c r="E1" s="9"/>
+      <c r="B1" s="11"/>
+      <c r="C1" s="11"/>
+      <c r="D1" s="11"/>
+      <c r="E1" s="11"/>
     </row>
     <row r="2" spans="1:7">
       <c r="A2" s="5" t="s">
@@ -3374,16 +3386,16 @@
       </c>
     </row>
     <row r="16" spans="1:7">
-      <c r="A16" s="10" t="s">
+      <c r="A16" s="12" t="s">
         <v>83</v>
       </c>
-      <c r="B16" s="11"/>
-      <c r="C16" s="12"/>
-      <c r="E16" s="10" t="s">
+      <c r="B16" s="13"/>
+      <c r="C16" s="14"/>
+      <c r="E16" s="12" t="s">
         <v>84</v>
       </c>
-      <c r="F16" s="11"/>
-      <c r="G16" s="12"/>
+      <c r="F16" s="13"/>
+      <c r="G16" s="14"/>
     </row>
     <row r="17" spans="1:7">
       <c r="A17" s="5" t="s">

</xml_diff>

<commit_message>
added the sql practive quesitons and snowflake 2.0
</commit_message>
<xml_diff>
--- a/05_Snowflake_Advance_DE_Certificate/Domain_Wise_Flow_Lost.xlsx
+++ b/05_Snowflake_Advance_DE_Certificate/Domain_Wise_Flow_Lost.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Snowflake_Advance_Data_Engineering\05_Snowflake_Advance_DE_Certificate\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{66356C77-D32E-4BD7-BA6F-D59DEA1C42D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7A7B0368-75AB-4AC4-91AF-B562BBE7A9E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="592" uniqueCount="240">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="593" uniqueCount="241">
   <si>
     <t>Step</t>
   </si>
@@ -1237,6 +1237,9 @@
   </si>
   <si>
     <t>🧠 Snowflake Advanced Data Engineer – Domain 1 (Data Movement) 14-Day Plan</t>
+  </si>
+  <si>
+    <t>explain these 2 topics in details with all explanation from scratch with syntax and examples in details to know for the advance snow pro core certification and admin should know about all these</t>
   </si>
 </sst>
 </file>
@@ -1879,6 +1882,9 @@
       </c>
     </row>
     <row r="15" spans="1:13">
+      <c r="E15" t="s">
+        <v>240</v>
+      </c>
       <c r="I15" s="16" t="s">
         <v>239</v>
       </c>
@@ -2435,13 +2441,13 @@
       <c r="C33" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="E33" s="3">
+      <c r="E33" s="9">
         <v>16</v>
       </c>
-      <c r="F33" s="4" t="s">
+      <c r="F33" s="9" t="s">
         <v>102</v>
       </c>
-      <c r="G33" s="3" t="s">
+      <c r="G33" s="9" t="s">
         <v>8</v>
       </c>
     </row>
@@ -2455,13 +2461,13 @@
       <c r="C34" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="E34" s="3">
-        <v>17</v>
-      </c>
-      <c r="F34" s="4" t="s">
+      <c r="E34" s="9">
+        <v>17</v>
+      </c>
+      <c r="F34" s="9" t="s">
         <v>103</v>
       </c>
-      <c r="G34" s="3" t="s">
+      <c r="G34" s="9" t="s">
         <v>8</v>
       </c>
     </row>

</xml_diff>